<commit_message>
Tighten action-column wrap and A3 print layout
Refit merged-column width and row heights so Chinese-then-English text wraps without clipped cells or oversized empty rows.

Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Action tracker - LILLY 按Area分类 中英对照 合并版 09-21-2026.xlsx
+++ b/Action tracker - LILLY 按Area分类 中英对照 合并版 09-21-2026.xlsx
@@ -13,6 +13,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'按Area分类（中英对照）'!$A$1:$K$67</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'按Area分类（中英对照）'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'按Area分类（中英对照）'!$A$1:$K$67</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -3680,7 +3681,7 @@
     <col width="11" customWidth="1" style="26" min="2" max="2"/>
     <col width="20" customWidth="1" style="26" min="3" max="3"/>
     <col width="22" customWidth="1" style="26" min="4" max="4"/>
-    <col width="50" customWidth="1" style="26" min="5" max="5"/>
+    <col width="52" customWidth="1" style="26" min="5" max="5"/>
     <col width="10" customWidth="1" style="26" min="6" max="6"/>
     <col width="22" customWidth="1" style="26" min="7" max="7"/>
     <col width="9" customWidth="1" style="26" min="8" max="8"/>
@@ -3689,7 +3690,7 @@
     <col width="24" customWidth="1" style="26" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42.4" customHeight="1" s="26">
+    <row r="1" ht="39.2" customHeight="1" s="26">
       <c r="A1" s="15" t="inlineStr">
         <is>
           <t>ID</t>
@@ -3771,7 +3772,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="50.8" customHeight="1" s="26">
+    <row r="2" ht="32.6" customHeight="1" s="26">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>BLA-025</t>
@@ -3832,7 +3833,7 @@
       <c r="J2" s="28" t="n"/>
       <c r="K2" s="28" t="n"/>
     </row>
-    <row r="3" ht="36.2" customHeight="1" s="26">
+    <row r="3" ht="32.6" customHeight="1" s="26">
       <c r="A3" s="29" t="inlineStr">
         <is>
           <t>BLA-009</t>
@@ -3893,7 +3894,7 @@
       <c r="J3" s="30" t="n"/>
       <c r="K3" s="30" t="n"/>
     </row>
-    <row r="4" ht="80" customHeight="1" s="26">
+    <row r="4" ht="60.2" customHeight="1" s="26">
       <c r="A4" s="29" t="inlineStr">
         <is>
           <t>BLA-104</t>
@@ -3959,7 +3960,7 @@
       </c>
       <c r="K4" s="30" t="n"/>
     </row>
-    <row r="5" ht="94.59999999999999" customHeight="1" s="26">
+    <row r="5" ht="74" customHeight="1" s="26">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>BLA-105</t>
@@ -4025,7 +4026,7 @@
       </c>
       <c r="K5" s="28" t="n"/>
     </row>
-    <row r="6" ht="109.2" customHeight="1" s="26">
+    <row r="6" ht="74" customHeight="1" s="26">
       <c r="A6" s="29" t="inlineStr">
         <is>
           <t>BLA-100</t>
@@ -4091,7 +4092,7 @@
       </c>
       <c r="K6" s="30" t="n"/>
     </row>
-    <row r="7" ht="109.2" customHeight="1" s="26">
+    <row r="7" ht="74" customHeight="1" s="26">
       <c r="A7" s="27" t="inlineStr">
         <is>
           <t>BLA-070</t>
@@ -4157,7 +4158,7 @@
       </c>
       <c r="K7" s="28" t="n"/>
     </row>
-    <row r="8" ht="153" customHeight="1" s="26">
+    <row r="8" ht="115.4" customHeight="1" s="26">
       <c r="A8" s="27" t="inlineStr">
         <is>
           <t>BLA-085</t>
@@ -4223,7 +4224,7 @@
       </c>
       <c r="K8" s="28" t="n"/>
     </row>
-    <row r="9" ht="109.2" customHeight="1" s="26">
+    <row r="9" ht="87.80000000000001" customHeight="1" s="26">
       <c r="A9" s="29" t="inlineStr">
         <is>
           <t>BLA-096</t>
@@ -4289,7 +4290,7 @@
       </c>
       <c r="K9" s="30" t="n"/>
     </row>
-    <row r="10" ht="211.4" customHeight="1" s="26">
+    <row r="10" ht="184.4" customHeight="1" s="26">
       <c r="A10" s="27" t="inlineStr">
         <is>
           <t>BLA-004</t>
@@ -4355,7 +4356,7 @@
       </c>
       <c r="K10" s="28" t="n"/>
     </row>
-    <row r="11" ht="123.8" customHeight="1" s="26">
+    <row r="11" ht="101.6" customHeight="1" s="26">
       <c r="A11" s="27" t="inlineStr">
         <is>
           <t>BLA-098</t>
@@ -4421,7 +4422,7 @@
       </c>
       <c r="K11" s="28" t="n"/>
     </row>
-    <row r="12" ht="80" customHeight="1" s="26">
+    <row r="12" ht="74" customHeight="1" s="26">
       <c r="A12" s="29" t="inlineStr">
         <is>
           <t>BLA-108</t>
@@ -4487,7 +4488,7 @@
       </c>
       <c r="K12" s="30" t="n"/>
     </row>
-    <row r="13" ht="94.59999999999999" customHeight="1" s="26">
+    <row r="13" ht="74" customHeight="1" s="26">
       <c r="A13" s="27" t="inlineStr">
         <is>
           <t>BLA-012</t>
@@ -4553,7 +4554,7 @@
       </c>
       <c r="K13" s="28" t="n"/>
     </row>
-    <row r="14" ht="50.8" customHeight="1" s="26">
+    <row r="14" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A14" s="27" t="inlineStr">
         <is>
           <t>BLA-013</t>
@@ -4614,7 +4615,7 @@
       <c r="J14" s="28" t="n"/>
       <c r="K14" s="28" t="n"/>
     </row>
-    <row r="15" ht="342.8" customHeight="1" s="26">
+    <row r="15" ht="294.8" customHeight="1" s="26">
       <c r="A15" s="27" t="inlineStr">
         <is>
           <t>BLA-091</t>
@@ -4680,7 +4681,7 @@
       </c>
       <c r="K15" s="28" t="n"/>
     </row>
-    <row r="16" ht="123.8" customHeight="1" s="26">
+    <row r="16" ht="115.4" customHeight="1" s="26">
       <c r="A16" s="27" t="inlineStr">
         <is>
           <t>BLA-092</t>
@@ -4746,7 +4747,7 @@
       </c>
       <c r="K16" s="28" t="n"/>
     </row>
-    <row r="17" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="17" ht="60.2" customHeight="1" s="26">
       <c r="A17" s="29" t="inlineStr">
         <is>
           <t>BLA-083</t>
@@ -4812,7 +4813,7 @@
       </c>
       <c r="K17" s="30" t="n"/>
     </row>
-    <row r="18" ht="80" customHeight="1" s="26">
+    <row r="18" ht="74" customHeight="1" s="26">
       <c r="A18" s="27" t="inlineStr">
         <is>
           <t>BLA-035</t>
@@ -4873,7 +4874,7 @@
       <c r="J18" s="28" t="n"/>
       <c r="K18" s="28" t="n"/>
     </row>
-    <row r="19" ht="80" customHeight="1" s="26">
+    <row r="19" ht="60.2" customHeight="1" s="26">
       <c r="A19" s="29" t="inlineStr">
         <is>
           <t>BLA-103</t>
@@ -4939,7 +4940,7 @@
       </c>
       <c r="K19" s="30" t="n"/>
     </row>
-    <row r="20" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="20" ht="60.2" customHeight="1" s="26">
       <c r="A20" s="27" t="inlineStr">
         <is>
           <t>BLA-077</t>
@@ -5005,7 +5006,7 @@
       </c>
       <c r="K20" s="28" t="n"/>
     </row>
-    <row r="21" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="21" ht="60.2" customHeight="1" s="26">
       <c r="A21" s="27" t="inlineStr">
         <is>
           <t>BLA-078</t>
@@ -5071,7 +5072,7 @@
       </c>
       <c r="K21" s="28" t="n"/>
     </row>
-    <row r="22" ht="80" customHeight="1" s="26">
+    <row r="22" ht="60.2" customHeight="1" s="26">
       <c r="A22" s="27" t="inlineStr">
         <is>
           <t>BLA-079</t>
@@ -5137,7 +5138,7 @@
       </c>
       <c r="K22" s="28" t="n"/>
     </row>
-    <row r="23" ht="80" customHeight="1" s="26">
+    <row r="23" ht="74" customHeight="1" s="26">
       <c r="A23" s="27" t="inlineStr">
         <is>
           <t>BLA-080</t>
@@ -5203,7 +5204,7 @@
       </c>
       <c r="K23" s="28" t="n"/>
     </row>
-    <row r="24" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="24" ht="60.2" customHeight="1" s="26">
       <c r="A24" s="29" t="inlineStr">
         <is>
           <t>BLA-081</t>
@@ -5269,7 +5270,7 @@
       </c>
       <c r="K24" s="30" t="n"/>
     </row>
-    <row r="25" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="25" ht="60.2" customHeight="1" s="26">
       <c r="A25" s="27" t="inlineStr">
         <is>
           <t>BLA-099</t>
@@ -5335,7 +5336,7 @@
       </c>
       <c r="K25" s="28" t="n"/>
     </row>
-    <row r="26" ht="123.8" customHeight="1" s="26">
+    <row r="26" ht="87.80000000000001" customHeight="1" s="26">
       <c r="A26" s="29" t="inlineStr">
         <is>
           <t>BLA-056</t>
@@ -5401,7 +5402,7 @@
       </c>
       <c r="K26" s="30" t="n"/>
     </row>
-    <row r="27" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="27" ht="60.2" customHeight="1" s="26">
       <c r="A27" s="29" t="inlineStr">
         <is>
           <t>BLA-057</t>
@@ -5467,7 +5468,7 @@
       </c>
       <c r="K27" s="30" t="n"/>
     </row>
-    <row r="28" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="28" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A28" s="29" t="inlineStr">
         <is>
           <t>BLA-058</t>
@@ -5533,7 +5534,7 @@
       </c>
       <c r="K28" s="30" t="n"/>
     </row>
-    <row r="29" ht="50.8" customHeight="1" s="26">
+    <row r="29" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A29" s="29" t="inlineStr">
         <is>
           <t>BLA-059</t>
@@ -5602,7 +5603,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="50.8" customHeight="1" s="26">
+    <row r="30" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A30" s="29" t="inlineStr">
         <is>
           <t>BLA-060</t>
@@ -5671,7 +5672,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="31" ht="60.2" customHeight="1" s="26">
       <c r="A31" s="27" t="inlineStr">
         <is>
           <t>BLA-042</t>
@@ -5740,7 +5741,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="50.8" customHeight="1" s="26">
+    <row r="32" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A32" s="27" t="inlineStr">
         <is>
           <t>BLA-043</t>
@@ -5801,7 +5802,7 @@
       <c r="J32" s="28" t="n"/>
       <c r="K32" s="28" t="n"/>
     </row>
-    <row r="33" ht="50.8" customHeight="1" s="26">
+    <row r="33" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A33" s="27" t="inlineStr">
         <is>
           <t>BLA-044</t>
@@ -5862,7 +5863,7 @@
       <c r="J33" s="28" t="n"/>
       <c r="K33" s="28" t="n"/>
     </row>
-    <row r="34" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="34" ht="60.2" customHeight="1" s="26">
       <c r="A34" s="27" t="inlineStr">
         <is>
           <t>BLA-045</t>
@@ -5931,7 +5932,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="35" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A35" s="27" t="inlineStr">
         <is>
           <t>BLA-074</t>
@@ -6000,7 +6001,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="50.8" customHeight="1" s="26">
+    <row r="36" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A36" s="27" t="inlineStr">
         <is>
           <t>BLA-076</t>
@@ -6069,7 +6070,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="37" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A37" s="27" t="inlineStr">
         <is>
           <t>BLA-086</t>
@@ -6138,7 +6139,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="50.8" customHeight="1" s="26">
+    <row r="38" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A38" s="27" t="inlineStr">
         <is>
           <t>BLA-087</t>
@@ -6207,7 +6208,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="80" customHeight="1" s="26">
+    <row r="39" ht="60.2" customHeight="1" s="26">
       <c r="A39" s="27" t="inlineStr">
         <is>
           <t>BLA-106</t>
@@ -6276,7 +6277,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="40" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A40" s="29" t="inlineStr">
         <is>
           <t>BLA-051</t>
@@ -6345,7 +6346,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="50.8" customHeight="1" s="26">
+    <row r="41" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A41" s="29" t="inlineStr">
         <is>
           <t>BLA-052</t>
@@ -6414,7 +6415,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="42" ht="60.2" customHeight="1" s="26">
       <c r="A42" s="29" t="inlineStr">
         <is>
           <t>BLA-055</t>
@@ -6483,7 +6484,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="43" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A43" s="27" t="inlineStr">
         <is>
           <t>BLA-053</t>
@@ -6552,7 +6553,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="44" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A44" s="27" t="inlineStr">
         <is>
           <t>BLA-054</t>
@@ -6621,7 +6622,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="50.8" customHeight="1" s="26">
+    <row r="45" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A45" s="29" t="inlineStr">
         <is>
           <t>BLA-016</t>
@@ -6690,7 +6691,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="46" ht="60.2" customHeight="1" s="26">
       <c r="A46" s="29" t="inlineStr">
         <is>
           <t>BLA-021</t>
@@ -6751,7 +6752,7 @@
       <c r="J46" s="30" t="n"/>
       <c r="K46" s="30" t="n"/>
     </row>
-    <row r="47" ht="80" customHeight="1" s="26">
+    <row r="47" ht="60.2" customHeight="1" s="26">
       <c r="A47" s="29" t="inlineStr">
         <is>
           <t>BLA-022</t>
@@ -6812,7 +6813,7 @@
       <c r="J47" s="30" t="n"/>
       <c r="K47" s="30" t="n"/>
     </row>
-    <row r="48" ht="80" customHeight="1" s="26">
+    <row r="48" ht="74" customHeight="1" s="26">
       <c r="A48" s="27" t="inlineStr">
         <is>
           <t>BLA-102</t>
@@ -6881,7 +6882,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="94.59999999999999" customHeight="1" s="26">
+    <row r="49" ht="87.80000000000001" customHeight="1" s="26">
       <c r="A49" s="29" t="inlineStr">
         <is>
           <t>BLA-097</t>
@@ -6950,7 +6951,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="109.2" customHeight="1" s="26">
+    <row r="50" ht="101.6" customHeight="1" s="26">
       <c r="A50" s="27" t="inlineStr">
         <is>
           <t>BLA-088</t>
@@ -7019,7 +7020,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="94.59999999999999" customHeight="1" s="26">
+    <row r="51" ht="74" customHeight="1" s="26">
       <c r="A51" s="27" t="inlineStr">
         <is>
           <t>BLA-089</t>
@@ -7088,7 +7089,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="94.59999999999999" customHeight="1" s="26">
+    <row r="52" ht="87.80000000000001" customHeight="1" s="26">
       <c r="A52" s="27" t="inlineStr">
         <is>
           <t>BLA-090</t>
@@ -7157,7 +7158,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="50.8" customHeight="1" s="26">
+    <row r="53" ht="32.6" customHeight="1" s="26">
       <c r="A53" s="29" t="inlineStr">
         <is>
           <t>BLA-061</t>
@@ -7226,7 +7227,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="54" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A54" s="29" t="inlineStr">
         <is>
           <t>BLA-062</t>
@@ -7295,7 +7296,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="50.8" customHeight="1" s="26">
+    <row r="55" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A55" s="29" t="inlineStr">
         <is>
           <t>BLA-063</t>
@@ -7364,7 +7365,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="50.8" customHeight="1" s="26">
+    <row r="56" ht="32.6" customHeight="1" s="26">
       <c r="A56" s="27" t="inlineStr">
         <is>
           <t>BLA-011</t>
@@ -7425,7 +7426,7 @@
       <c r="J56" s="28" t="n"/>
       <c r="K56" s="28" t="n"/>
     </row>
-    <row r="57" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="57" ht="60.2" customHeight="1" s="26">
       <c r="A57" s="29" t="inlineStr">
         <is>
           <t>BLA-110</t>
@@ -7494,7 +7495,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="269.8" customHeight="1" s="26">
+    <row r="58" ht="225.8" customHeight="1" s="26">
       <c r="A58" s="27" t="inlineStr">
         <is>
           <t>BLA-093</t>
@@ -7563,7 +7564,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="80" customHeight="1" s="26">
+    <row r="59" ht="74" customHeight="1" s="26">
       <c r="A59" s="27" t="inlineStr">
         <is>
           <t>BLA-094</t>
@@ -7632,7 +7633,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="94.59999999999999" customHeight="1" s="26">
+    <row r="60" ht="74" customHeight="1" s="26">
       <c r="A60" s="27" t="inlineStr">
         <is>
           <t>BLA-095</t>
@@ -7701,7 +7702,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="80" customHeight="1" s="26">
+    <row r="61" ht="74" customHeight="1" s="26">
       <c r="A61" s="29" t="inlineStr">
         <is>
           <t>BLA-065</t>
@@ -7770,7 +7771,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="62" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A62" s="29" t="inlineStr">
         <is>
           <t>BLA-066</t>
@@ -7839,7 +7840,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="109.2" customHeight="1" s="26">
+    <row r="63" ht="101.6" customHeight="1" s="26">
       <c r="A63" s="27" t="inlineStr">
         <is>
           <t>BLA-107</t>
@@ -7908,7 +7909,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="50.8" customHeight="1" s="26">
+    <row r="64" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A64" s="29" t="inlineStr">
         <is>
           <t>BLA-109</t>
@@ -7977,7 +7978,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="109.2" customHeight="1" s="26">
+    <row r="65" ht="87.80000000000001" customHeight="1" s="26">
       <c r="A65" s="27" t="inlineStr">
         <is>
           <t>BLA-101</t>
@@ -8046,7 +8047,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="65.40000000000001" customHeight="1" s="26">
+    <row r="66" ht="46.40000000000001" customHeight="1" s="26">
       <c r="A66" s="29" t="inlineStr">
         <is>
           <t>BLA-084</t>
@@ -8115,7 +8116,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="80" customHeight="1" s="26">
+    <row r="67" ht="74" customHeight="1" s="26">
       <c r="A67" s="27" t="inlineStr">
         <is>
           <t>BLA-111</t>

</xml_diff>